<commit_message>
data: add Sweet Lands and relocate Set a Watch
</commit_message>
<xml_diff>
--- a/game-system/game-data/source/2-cottage-manual/cottage-owned-games.xlsx
+++ b/game-system/game-data/source/2-cottage-manual/cottage-owned-games.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4152" uniqueCount="1357">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4154" uniqueCount="1359">
   <si>
     <t xml:space="preserve"> &lt;필터 바꾸셔도 됩니다&gt;</t>
   </si>
@@ -3627,6 +3627,9 @@
     <t>파수꾼</t>
   </si>
   <si>
+    <t>쉬운 협력</t>
+  </si>
+  <si>
     <t>파수꾼들</t>
   </si>
   <si>
@@ -4009,6 +4012,9 @@
   </si>
   <si>
     <t>아르낙의잊혀진유적</t>
+  </si>
+  <si>
+    <t>스위트랜드</t>
   </si>
   <si>
     <t>보유게임리스트는 탭을 이동해주세요</t>
@@ -5359,7 +5365,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AB1053"/>
+  <dimension ref="A1:AB1054"/>
   <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="12.63" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.38" customWidth="1"/>
@@ -24878,7 +24884,7 @@
         <v>2.43</v>
       </c>
       <c r="C577" s="20" t="s">
-        <v>421</v>
+        <v>1192</v>
       </c>
       <c r="D577" s="21" t="s">
         <v>615</v>
@@ -24887,16 +24893,16 @@
         <v>7.2</v>
       </c>
       <c r="F577" s="64" t="s">
-        <v>1192</v>
+        <v>1193</v>
       </c>
       <c r="G577" s="25" t="s">
-        <v>1192</v>
+        <v>1193</v>
       </c>
       <c r="H577" s="25" t="s">
-        <v>1192</v>
+        <v>1193</v>
       </c>
       <c r="I577" s="25" t="s">
-        <v>1192</v>
+        <v>1193</v>
       </c>
       <c r="J577" s="24"/>
       <c r="K577" s="24"/>
@@ -24909,7 +24915,7 @@
     </row>
     <row r="578" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A578" s="18" t="s">
-        <v>1193</v>
+        <v>1194</v>
       </c>
       <c r="B578" s="19">
         <v>3.85</v>
@@ -24922,19 +24928,19 @@
         <v>8.1</v>
       </c>
       <c r="F578" s="27" t="s">
-        <v>1194</v>
+        <v>1195</v>
       </c>
       <c r="G578" s="25" t="s">
-        <v>1194</v>
+        <v>1195</v>
       </c>
       <c r="H578" s="25" t="s">
-        <v>1194</v>
+        <v>1195</v>
       </c>
       <c r="I578" s="25" t="s">
-        <v>1194</v>
+        <v>1195</v>
       </c>
       <c r="J578" s="25" t="s">
-        <v>1194</v>
+        <v>1195</v>
       </c>
       <c r="K578" s="24"/>
       <c r="L578" s="35"/>
@@ -24946,7 +24952,7 @@
     </row>
     <row r="579" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A579" s="18" t="s">
-        <v>1195</v>
+        <v>1196</v>
       </c>
       <c r="B579" s="19">
         <v>2.08</v>
@@ -24955,16 +24961,16 @@
         <v>172</v>
       </c>
       <c r="D579" s="21" t="s">
-        <v>1196</v>
+        <v>1197</v>
       </c>
       <c r="E579" s="22">
         <v>6.7</v>
       </c>
       <c r="F579" s="64" t="s">
-        <v>1197</v>
+        <v>1198</v>
       </c>
       <c r="G579" s="25" t="s">
-        <v>1197</v>
+        <v>1198</v>
       </c>
       <c r="H579" s="24"/>
       <c r="I579" s="24"/>
@@ -24977,7 +24983,7 @@
     </row>
     <row r="580" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A580" s="18" t="s">
-        <v>1198</v>
+        <v>1199</v>
       </c>
       <c r="B580" s="43">
         <v>1.81</v>
@@ -24986,23 +24992,23 @@
         <v>18</v>
       </c>
       <c r="D580" s="21" t="s">
-        <v>1199</v>
+        <v>1200</v>
       </c>
       <c r="E580" s="22">
         <v>7.5</v>
       </c>
       <c r="F580" s="23"/>
       <c r="G580" s="25" t="s">
-        <v>1200</v>
+        <v>1201</v>
       </c>
       <c r="H580" s="25" t="s">
-        <v>1200</v>
+        <v>1201</v>
       </c>
       <c r="I580" s="25" t="s">
-        <v>1200</v>
+        <v>1201</v>
       </c>
       <c r="J580" s="25" t="s">
-        <v>1200</v>
+        <v>1201</v>
       </c>
       <c r="K580" s="24"/>
       <c r="L580" s="24"/>
@@ -25012,7 +25018,7 @@
     </row>
     <row r="581" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A581" s="18" t="s">
-        <v>1201</v>
+        <v>1202</v>
       </c>
       <c r="B581" s="19">
         <v>2.63</v>
@@ -25027,16 +25033,16 @@
         <v>7.7</v>
       </c>
       <c r="F581" s="40" t="s">
-        <v>1201</v>
+        <v>1202</v>
       </c>
       <c r="G581" s="31" t="s">
-        <v>1201</v>
+        <v>1202</v>
       </c>
       <c r="H581" s="31" t="s">
-        <v>1201</v>
+        <v>1202</v>
       </c>
       <c r="I581" s="30" t="s">
-        <v>1201</v>
+        <v>1202</v>
       </c>
       <c r="J581" s="24"/>
       <c r="K581" s="24"/>
@@ -25047,7 +25053,7 @@
     </row>
     <row r="582" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A582" s="18" t="s">
-        <v>1202</v>
+        <v>1203</v>
       </c>
       <c r="B582" s="19">
         <v>1.6</v>
@@ -25063,7 +25069,7 @@
       </c>
       <c r="F582" s="23"/>
       <c r="G582" s="25" t="s">
-        <v>1203</v>
+        <v>1204</v>
       </c>
       <c r="H582" s="24"/>
       <c r="I582" s="24"/>
@@ -25076,7 +25082,7 @@
     </row>
     <row r="583" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A583" s="18" t="s">
-        <v>1204</v>
+        <v>1205</v>
       </c>
       <c r="B583" s="19">
         <v>2.4</v>
@@ -25091,16 +25097,16 @@
         <v>7.5</v>
       </c>
       <c r="F583" s="27" t="s">
-        <v>1205</v>
+        <v>1206</v>
       </c>
       <c r="G583" s="25" t="s">
-        <v>1205</v>
+        <v>1206</v>
       </c>
       <c r="H583" s="25" t="s">
-        <v>1205</v>
+        <v>1206</v>
       </c>
       <c r="I583" s="25" t="s">
-        <v>1205</v>
+        <v>1206</v>
       </c>
       <c r="J583" s="24"/>
       <c r="K583" s="24"/>
@@ -25111,7 +25117,7 @@
     </row>
     <row r="584" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A584" s="18" t="s">
-        <v>1206</v>
+        <v>1207</v>
       </c>
       <c r="B584" s="19">
         <v>2.41</v>
@@ -25125,13 +25131,13 @@
       </c>
       <c r="F584" s="23"/>
       <c r="G584" s="25" t="s">
-        <v>1207</v>
+        <v>1208</v>
       </c>
       <c r="H584" s="25" t="s">
-        <v>1207</v>
+        <v>1208</v>
       </c>
       <c r="I584" s="25" t="s">
-        <v>1207</v>
+        <v>1208</v>
       </c>
       <c r="J584" s="24"/>
       <c r="K584" s="24"/>
@@ -25144,7 +25150,7 @@
     </row>
     <row r="585" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A585" s="18" t="s">
-        <v>1208</v>
+        <v>1209</v>
       </c>
       <c r="B585" s="19">
         <v>2.8</v>
@@ -25153,20 +25159,20 @@
         <v>185</v>
       </c>
       <c r="D585" s="21" t="s">
-        <v>1209</v>
+        <v>1210</v>
       </c>
       <c r="E585" s="22">
         <v>7.4</v>
       </c>
       <c r="F585" s="23"/>
       <c r="G585" s="25" t="s">
-        <v>1210</v>
+        <v>1211</v>
       </c>
       <c r="H585" s="25" t="s">
-        <v>1210</v>
+        <v>1211</v>
       </c>
       <c r="I585" s="25" t="s">
-        <v>1210</v>
+        <v>1211</v>
       </c>
       <c r="J585" s="24"/>
       <c r="K585" s="24"/>
@@ -25179,7 +25185,7 @@
     </row>
     <row r="586" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A586" s="18" t="s">
-        <v>1211</v>
+        <v>1212</v>
       </c>
       <c r="B586" s="19">
         <v>3.35</v>
@@ -25193,13 +25199,13 @@
       </c>
       <c r="F586" s="23"/>
       <c r="G586" s="25" t="s">
-        <v>1211</v>
+        <v>1212</v>
       </c>
       <c r="H586" s="25" t="s">
-        <v>1211</v>
+        <v>1212</v>
       </c>
       <c r="I586" s="25" t="s">
-        <v>1211</v>
+        <v>1212</v>
       </c>
       <c r="J586" s="24"/>
       <c r="K586" s="24"/>
@@ -25212,7 +25218,7 @@
     </row>
     <row r="587" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A587" s="18" t="s">
-        <v>1212</v>
+        <v>1213</v>
       </c>
       <c r="B587" s="19">
         <v>3.08</v>
@@ -25227,10 +25233,10 @@
       <c r="F587" s="85"/>
       <c r="G587" s="35"/>
       <c r="H587" s="25" t="s">
-        <v>1212</v>
+        <v>1213</v>
       </c>
       <c r="I587" s="25" t="s">
-        <v>1212</v>
+        <v>1213</v>
       </c>
       <c r="J587" s="24"/>
       <c r="K587" s="24"/>
@@ -25243,7 +25249,7 @@
     </row>
     <row r="588" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A588" s="18" t="s">
-        <v>1213</v>
+        <v>1214</v>
       </c>
       <c r="B588" s="19">
         <v>1.2</v>
@@ -25252,7 +25258,7 @@
         <v>21</v>
       </c>
       <c r="D588" s="21" t="s">
-        <v>1214</v>
+        <v>1215</v>
       </c>
       <c r="E588" s="22">
         <v>6.8</v>
@@ -25260,13 +25266,13 @@
       <c r="F588" s="23"/>
       <c r="G588" s="25"/>
       <c r="H588" s="25" t="s">
-        <v>1215</v>
+        <v>1216</v>
       </c>
       <c r="I588" s="25" t="s">
-        <v>1215</v>
+        <v>1216</v>
       </c>
       <c r="J588" s="25" t="s">
-        <v>1215</v>
+        <v>1216</v>
       </c>
       <c r="K588" s="24"/>
       <c r="L588" s="24"/>
@@ -25276,7 +25282,7 @@
     </row>
     <row r="589" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A589" s="18" t="s">
-        <v>1216</v>
+        <v>1217</v>
       </c>
       <c r="B589" s="19">
         <v>1.2</v>
@@ -25293,13 +25299,13 @@
       <c r="F589" s="23"/>
       <c r="G589" s="25"/>
       <c r="H589" s="25" t="s">
-        <v>1215</v>
+        <v>1216</v>
       </c>
       <c r="I589" s="25" t="s">
-        <v>1215</v>
+        <v>1216</v>
       </c>
       <c r="J589" s="25" t="s">
-        <v>1215</v>
+        <v>1216</v>
       </c>
       <c r="K589" s="24"/>
       <c r="L589" s="24"/>
@@ -25309,13 +25315,13 @@
     </row>
     <row r="590" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A590" s="18" t="s">
-        <v>1217</v>
+        <v>1218</v>
       </c>
       <c r="B590" s="19" t="s">
         <v>29</v>
       </c>
       <c r="C590" s="20" t="s">
-        <v>1218</v>
+        <v>1219</v>
       </c>
       <c r="D590" s="21" t="s">
         <v>952</v>
@@ -25324,10 +25330,10 @@
         <v>7</v>
       </c>
       <c r="F590" s="27" t="s">
-        <v>1219</v>
+        <v>1220</v>
       </c>
       <c r="G590" s="25" t="s">
-        <v>1219</v>
+        <v>1220</v>
       </c>
       <c r="H590" s="24"/>
       <c r="I590" s="24"/>
@@ -25340,7 +25346,7 @@
     </row>
     <row r="591" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A591" s="18" t="s">
-        <v>1220</v>
+        <v>1221</v>
       </c>
       <c r="B591" s="19">
         <v>1.4</v>
@@ -25349,7 +25355,7 @@
         <v>26</v>
       </c>
       <c r="D591" s="21" t="s">
-        <v>1221</v>
+        <v>1222</v>
       </c>
       <c r="E591" s="22">
         <v>6.6</v>
@@ -25357,13 +25363,13 @@
       <c r="F591" s="27"/>
       <c r="G591" s="24"/>
       <c r="H591" s="30" t="s">
-        <v>1222</v>
+        <v>1223</v>
       </c>
       <c r="I591" s="30" t="s">
-        <v>1222</v>
+        <v>1223</v>
       </c>
       <c r="J591" s="31" t="s">
-        <v>1222</v>
+        <v>1223</v>
       </c>
       <c r="K591" s="24"/>
       <c r="L591" s="24"/>
@@ -25373,7 +25379,7 @@
     </row>
     <row r="592" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A592" s="18" t="s">
-        <v>1223</v>
+        <v>1224</v>
       </c>
       <c r="B592" s="19">
         <v>1</v>
@@ -25389,13 +25395,13 @@
       </c>
       <c r="F592" s="23"/>
       <c r="G592" s="25" t="s">
-        <v>1224</v>
+        <v>1225</v>
       </c>
       <c r="H592" s="25" t="s">
-        <v>1224</v>
+        <v>1225</v>
       </c>
       <c r="I592" s="25" t="s">
-        <v>1224</v>
+        <v>1225</v>
       </c>
       <c r="J592" s="24"/>
       <c r="K592" s="24"/>
@@ -25406,7 +25412,7 @@
     </row>
     <row r="593" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A593" s="18" t="s">
-        <v>1225</v>
+        <v>1226</v>
       </c>
       <c r="B593" s="19">
         <v>2.21</v>
@@ -25422,13 +25428,13 @@
       </c>
       <c r="F593" s="23"/>
       <c r="G593" s="25" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="H593" s="25" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="I593" s="25" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="J593" s="24"/>
       <c r="K593" s="24"/>
@@ -25439,7 +25445,7 @@
     </row>
     <row r="594" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A594" s="18" t="s">
-        <v>1227</v>
+        <v>1228</v>
       </c>
       <c r="B594" s="19">
         <v>2.04</v>
@@ -25452,19 +25458,19 @@
         <v>7.1</v>
       </c>
       <c r="F594" s="27" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
       <c r="G594" s="25" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
       <c r="H594" s="25" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
       <c r="I594" s="25" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
       <c r="J594" s="25" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
       <c r="K594" s="24"/>
       <c r="L594" s="24"/>
@@ -25474,7 +25480,7 @@
     </row>
     <row r="595" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A595" s="18" t="s">
-        <v>1229</v>
+        <v>1230</v>
       </c>
       <c r="B595" s="32">
         <v>1.73</v>
@@ -25483,22 +25489,22 @@
         <v>172</v>
       </c>
       <c r="D595" s="21" t="s">
-        <v>1230</v>
+        <v>1231</v>
       </c>
       <c r="E595" s="22">
         <v>6.8</v>
       </c>
       <c r="F595" s="27" t="s">
-        <v>1231</v>
+        <v>1232</v>
       </c>
       <c r="G595" s="25" t="s">
-        <v>1231</v>
+        <v>1232</v>
       </c>
       <c r="H595" s="25" t="s">
-        <v>1231</v>
+        <v>1232</v>
       </c>
       <c r="I595" s="25" t="s">
-        <v>1231</v>
+        <v>1232</v>
       </c>
       <c r="J595" s="24"/>
       <c r="K595" s="24"/>
@@ -25509,7 +25515,7 @@
     </row>
     <row r="596" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A596" s="18" t="s">
-        <v>1232</v>
+        <v>1233</v>
       </c>
       <c r="B596" s="43">
         <v>1.77</v>
@@ -25518,20 +25524,20 @@
         <v>18</v>
       </c>
       <c r="D596" s="21" t="s">
-        <v>1233</v>
+        <v>1234</v>
       </c>
       <c r="E596" s="22">
         <v>7.1</v>
       </c>
       <c r="F596" s="23"/>
       <c r="G596" s="25" t="s">
-        <v>1234</v>
+        <v>1235</v>
       </c>
       <c r="H596" s="25" t="s">
-        <v>1234</v>
+        <v>1235</v>
       </c>
       <c r="I596" s="25" t="s">
-        <v>1234</v>
+        <v>1235</v>
       </c>
       <c r="J596" s="24"/>
       <c r="K596" s="24"/>
@@ -25542,7 +25548,7 @@
     </row>
     <row r="597" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A597" s="18" t="s">
-        <v>1235</v>
+        <v>1236</v>
       </c>
       <c r="B597" s="19">
         <v>1.44</v>
@@ -25557,16 +25563,16 @@
         <v>6.7</v>
       </c>
       <c r="F597" s="27" t="s">
-        <v>1236</v>
+        <v>1237</v>
       </c>
       <c r="G597" s="25" t="s">
-        <v>1236</v>
+        <v>1237</v>
       </c>
       <c r="H597" s="25" t="s">
-        <v>1236</v>
+        <v>1237</v>
       </c>
       <c r="I597" s="25" t="s">
-        <v>1236</v>
+        <v>1237</v>
       </c>
       <c r="J597" s="24"/>
       <c r="K597" s="24"/>
@@ -25579,7 +25585,7 @@
     </row>
     <row r="598" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A598" s="18" t="s">
-        <v>1237</v>
+        <v>1238</v>
       </c>
       <c r="B598" s="19">
         <v>1</v>
@@ -25608,7 +25614,7 @@
     </row>
     <row r="599" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A599" s="18" t="s">
-        <v>1238</v>
+        <v>1239</v>
       </c>
       <c r="B599" s="19">
         <v>1.61</v>
@@ -25617,23 +25623,23 @@
         <v>18</v>
       </c>
       <c r="D599" s="21" t="s">
-        <v>1239</v>
+        <v>1240</v>
       </c>
       <c r="E599" s="22">
         <v>7.1</v>
       </c>
       <c r="F599" s="23"/>
       <c r="G599" s="25" t="s">
-        <v>1238</v>
+        <v>1239</v>
       </c>
       <c r="H599" s="25" t="s">
-        <v>1238</v>
+        <v>1239</v>
       </c>
       <c r="I599" s="25" t="s">
-        <v>1238</v>
+        <v>1239</v>
       </c>
       <c r="J599" s="25" t="s">
-        <v>1238</v>
+        <v>1239</v>
       </c>
       <c r="K599" s="24"/>
       <c r="L599" s="24"/>
@@ -25643,7 +25649,7 @@
     </row>
     <row r="600" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A600" s="18" t="s">
-        <v>1240</v>
+        <v>1241</v>
       </c>
       <c r="B600" s="19">
         <v>1</v>
@@ -25658,19 +25664,19 @@
         <v>7.2</v>
       </c>
       <c r="F600" s="40" t="s">
-        <v>1240</v>
+        <v>1241</v>
       </c>
       <c r="G600" s="31" t="s">
-        <v>1240</v>
+        <v>1241</v>
       </c>
       <c r="H600" s="31" t="s">
-        <v>1240</v>
+        <v>1241</v>
       </c>
       <c r="I600" s="31" t="s">
-        <v>1240</v>
+        <v>1241</v>
       </c>
       <c r="J600" s="31" t="s">
-        <v>1240</v>
+        <v>1241</v>
       </c>
       <c r="K600" s="24"/>
       <c r="L600" s="24"/>
@@ -25680,7 +25686,7 @@
     </row>
     <row r="601" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A601" s="18" t="s">
-        <v>1241</v>
+        <v>1242</v>
       </c>
       <c r="B601" s="19">
         <v>1</v>
@@ -25705,7 +25711,7 @@
     </row>
     <row r="602" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A602" s="18" t="s">
-        <v>1242</v>
+        <v>1243</v>
       </c>
       <c r="B602" s="19">
         <v>3.25</v>
@@ -25721,16 +25727,16 @@
       </c>
       <c r="F602" s="23"/>
       <c r="G602" s="25" t="s">
-        <v>1243</v>
+        <v>1244</v>
       </c>
       <c r="H602" s="25" t="s">
-        <v>1243</v>
+        <v>1244</v>
       </c>
       <c r="I602" s="25" t="s">
-        <v>1243</v>
+        <v>1244</v>
       </c>
       <c r="J602" s="25" t="s">
-        <v>1243</v>
+        <v>1244</v>
       </c>
       <c r="K602" s="24"/>
       <c r="L602" s="24"/>
@@ -25740,7 +25746,7 @@
     </row>
     <row r="603" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A603" s="18" t="s">
-        <v>1244</v>
+        <v>1245</v>
       </c>
       <c r="B603" s="19">
         <v>3.84</v>
@@ -25749,22 +25755,22 @@
         <v>421</v>
       </c>
       <c r="D603" s="21" t="s">
-        <v>1245</v>
+        <v>1246</v>
       </c>
       <c r="E603" s="22">
         <v>8.6</v>
       </c>
       <c r="F603" s="27" t="s">
-        <v>1246</v>
+        <v>1247</v>
       </c>
       <c r="G603" s="25" t="s">
-        <v>1246</v>
+        <v>1247</v>
       </c>
       <c r="H603" s="25" t="s">
-        <v>1246</v>
+        <v>1247</v>
       </c>
       <c r="I603" s="25" t="s">
-        <v>1246</v>
+        <v>1247</v>
       </c>
       <c r="J603" s="24"/>
       <c r="K603" s="24"/>
@@ -25777,7 +25783,7 @@
     </row>
     <row r="604" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A604" s="18" t="s">
-        <v>1247</v>
+        <v>1248</v>
       </c>
       <c r="B604" s="19">
         <v>2.64</v>
@@ -25793,13 +25799,13 @@
       </c>
       <c r="F604" s="23"/>
       <c r="G604" s="25" t="s">
-        <v>1247</v>
+        <v>1248</v>
       </c>
       <c r="H604" s="25" t="s">
-        <v>1247</v>
+        <v>1248</v>
       </c>
       <c r="I604" s="25" t="s">
-        <v>1247</v>
+        <v>1248</v>
       </c>
       <c r="J604" s="24"/>
       <c r="K604" s="24"/>
@@ -25810,7 +25816,7 @@
     </row>
     <row r="605" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A605" s="18" t="s">
-        <v>1248</v>
+        <v>1249</v>
       </c>
       <c r="B605" s="19">
         <v>1.56</v>
@@ -25825,16 +25831,16 @@
         <v>7.5</v>
       </c>
       <c r="F605" s="40" t="s">
-        <v>1248</v>
+        <v>1249</v>
       </c>
       <c r="G605" s="31" t="s">
-        <v>1248</v>
+        <v>1249</v>
       </c>
       <c r="H605" s="31" t="s">
-        <v>1248</v>
+        <v>1249</v>
       </c>
       <c r="I605" s="30" t="s">
-        <v>1248</v>
+        <v>1249</v>
       </c>
       <c r="J605" s="24"/>
       <c r="K605" s="24"/>
@@ -25845,7 +25851,7 @@
     </row>
     <row r="606" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A606" s="18" t="s">
-        <v>1249</v>
+        <v>1250</v>
       </c>
       <c r="B606" s="19">
         <v>2.41</v>
@@ -25854,22 +25860,22 @@
         <v>18</v>
       </c>
       <c r="D606" s="21" t="s">
-        <v>1250</v>
+        <v>1251</v>
       </c>
       <c r="E606" s="22">
         <v>7.8</v>
       </c>
       <c r="F606" s="23" t="s">
-        <v>1249</v>
+        <v>1250</v>
       </c>
       <c r="G606" s="25" t="s">
-        <v>1249</v>
+        <v>1250</v>
       </c>
       <c r="H606" s="25" t="s">
-        <v>1249</v>
+        <v>1250</v>
       </c>
       <c r="I606" s="25" t="s">
-        <v>1249</v>
+        <v>1250</v>
       </c>
       <c r="J606" s="24"/>
       <c r="K606" s="51"/>
@@ -25879,7 +25885,7 @@
     </row>
     <row r="607" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A607" s="18" t="s">
-        <v>1251</v>
+        <v>1252</v>
       </c>
       <c r="B607" s="19">
         <v>3.24</v>
@@ -25896,13 +25902,13 @@
       <c r="F607" s="23"/>
       <c r="G607" s="24"/>
       <c r="H607" s="25" t="s">
-        <v>1252</v>
+        <v>1253</v>
       </c>
       <c r="I607" s="25" t="s">
-        <v>1252</v>
+        <v>1253</v>
       </c>
       <c r="J607" s="25" t="s">
-        <v>1252</v>
+        <v>1253</v>
       </c>
       <c r="K607" s="24"/>
       <c r="L607" s="24"/>
@@ -25912,7 +25918,7 @@
     </row>
     <row r="608" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A608" s="18" t="s">
-        <v>1253</v>
+        <v>1254</v>
       </c>
       <c r="B608" s="19">
         <v>2.08</v>
@@ -25928,13 +25934,13 @@
       </c>
       <c r="F608" s="23"/>
       <c r="G608" s="31" t="s">
-        <v>1253</v>
+        <v>1254</v>
       </c>
       <c r="H608" s="31" t="s">
-        <v>1253</v>
+        <v>1254</v>
       </c>
       <c r="I608" s="30" t="s">
-        <v>1253</v>
+        <v>1254</v>
       </c>
       <c r="J608" s="24"/>
       <c r="K608" s="24"/>
@@ -25945,7 +25951,7 @@
     </row>
     <row r="609" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A609" s="18" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="B609" s="19">
         <v>2.03</v>
@@ -25959,13 +25965,13 @@
       </c>
       <c r="F609" s="23"/>
       <c r="G609" s="25" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="H609" s="25" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="I609" s="25" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="J609" s="24"/>
       <c r="K609" s="24"/>
@@ -25978,7 +25984,7 @@
     </row>
     <row r="610" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A610" s="18" t="s">
-        <v>1256</v>
+        <v>1257</v>
       </c>
       <c r="B610" s="19">
         <v>1.68</v>
@@ -25992,7 +25998,7 @@
       </c>
       <c r="F610" s="23"/>
       <c r="G610" s="25" t="s">
-        <v>1257</v>
+        <v>1258</v>
       </c>
       <c r="H610" s="24"/>
       <c r="I610" s="24"/>
@@ -26005,7 +26011,7 @@
     </row>
     <row r="611" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A611" s="18" t="s">
-        <v>1258</v>
+        <v>1259</v>
       </c>
       <c r="B611" s="19">
         <v>2.07</v>
@@ -26021,16 +26027,16 @@
       </c>
       <c r="F611" s="23"/>
       <c r="G611" s="25" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
       <c r="H611" s="25" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
       <c r="I611" s="25" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
       <c r="J611" s="25" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
       <c r="K611" s="24"/>
       <c r="L611" s="24"/>
@@ -26040,7 +26046,7 @@
     </row>
     <row r="612" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A612" s="18" t="s">
-        <v>1260</v>
+        <v>1261</v>
       </c>
       <c r="B612" s="32">
         <v>2.21</v>
@@ -26056,16 +26062,16 @@
       </c>
       <c r="F612" s="23"/>
       <c r="G612" s="30" t="s">
-        <v>1260</v>
+        <v>1261</v>
       </c>
       <c r="H612" s="30" t="s">
-        <v>1260</v>
+        <v>1261</v>
       </c>
       <c r="I612" s="31" t="s">
-        <v>1260</v>
+        <v>1261</v>
       </c>
       <c r="J612" s="31" t="s">
-        <v>1260</v>
+        <v>1261</v>
       </c>
       <c r="K612" s="24"/>
       <c r="L612" s="24"/>
@@ -26075,7 +26081,7 @@
     </row>
     <row r="613" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A613" s="18" t="s">
-        <v>1261</v>
+        <v>1262</v>
       </c>
       <c r="B613" s="19">
         <v>3.15</v>
@@ -26090,13 +26096,13 @@
         <v>7.9</v>
       </c>
       <c r="F613" s="64" t="s">
-        <v>1262</v>
+        <v>1263</v>
       </c>
       <c r="G613" s="25" t="s">
-        <v>1262</v>
+        <v>1263</v>
       </c>
       <c r="H613" s="25" t="s">
-        <v>1262</v>
+        <v>1263</v>
       </c>
       <c r="I613" s="24"/>
       <c r="J613" s="24"/>
@@ -26108,7 +26114,7 @@
     </row>
     <row r="614" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A614" s="18" t="s">
-        <v>1263</v>
+        <v>1264</v>
       </c>
       <c r="B614" s="19">
         <v>2.01</v>
@@ -26123,16 +26129,16 @@
         <v>8</v>
       </c>
       <c r="F614" s="27" t="s">
-        <v>1263</v>
+        <v>1264</v>
       </c>
       <c r="G614" s="25" t="s">
-        <v>1263</v>
+        <v>1264</v>
       </c>
       <c r="H614" s="25" t="s">
-        <v>1263</v>
+        <v>1264</v>
       </c>
       <c r="I614" s="25" t="s">
-        <v>1263</v>
+        <v>1264</v>
       </c>
       <c r="J614" s="24"/>
       <c r="K614" s="24"/>
@@ -26143,7 +26149,7 @@
     </row>
     <row r="615" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A615" s="18" t="s">
-        <v>1264</v>
+        <v>1265</v>
       </c>
       <c r="B615" s="19">
         <v>2.31</v>
@@ -26159,7 +26165,7 @@
       </c>
       <c r="F615" s="23"/>
       <c r="G615" s="25" t="s">
-        <v>1264</v>
+        <v>1265</v>
       </c>
       <c r="H615" s="24"/>
       <c r="I615" s="24"/>
@@ -26172,7 +26178,7 @@
     </row>
     <row r="616" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A616" s="18" t="s">
-        <v>1265</v>
+        <v>1266</v>
       </c>
       <c r="B616" s="19">
         <v>1.48</v>
@@ -26189,13 +26195,13 @@
       <c r="F616" s="23"/>
       <c r="G616" s="24"/>
       <c r="H616" s="25" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="I616" s="25" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="J616" s="25" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="K616" s="24"/>
       <c r="L616" s="24"/>
@@ -26205,7 +26211,7 @@
     </row>
     <row r="617" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A617" s="18" t="s">
-        <v>1267</v>
+        <v>1268</v>
       </c>
       <c r="B617" s="19">
         <v>2.54</v>
@@ -26221,13 +26227,13 @@
       </c>
       <c r="F617" s="23"/>
       <c r="G617" s="25" t="s">
-        <v>1268</v>
+        <v>1269</v>
       </c>
       <c r="H617" s="25" t="s">
-        <v>1268</v>
+        <v>1269</v>
       </c>
       <c r="I617" s="25" t="s">
-        <v>1268</v>
+        <v>1269</v>
       </c>
       <c r="J617" s="24"/>
       <c r="K617" s="24"/>
@@ -26238,7 +26244,7 @@
     </row>
     <row r="618" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A618" s="18" t="s">
-        <v>1269</v>
+        <v>1270</v>
       </c>
       <c r="B618" s="19">
         <v>2.95</v>
@@ -26255,13 +26261,13 @@
       <c r="F618" s="23"/>
       <c r="G618" s="27"/>
       <c r="H618" s="25" t="s">
-        <v>1270</v>
+        <v>1271</v>
       </c>
       <c r="I618" s="25" t="s">
-        <v>1270</v>
+        <v>1271</v>
       </c>
       <c r="J618" s="25" t="s">
-        <v>1270</v>
+        <v>1271</v>
       </c>
       <c r="K618" s="24"/>
       <c r="L618" s="24"/>
@@ -26271,7 +26277,7 @@
     </row>
     <row r="619" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A619" s="18" t="s">
-        <v>1271</v>
+        <v>1272</v>
       </c>
       <c r="B619" s="19">
         <v>3.3</v>
@@ -26286,16 +26292,16 @@
         <v>7.8</v>
       </c>
       <c r="F619" s="27" t="s">
-        <v>1271</v>
+        <v>1272</v>
       </c>
       <c r="G619" s="25" t="s">
-        <v>1271</v>
+        <v>1272</v>
       </c>
       <c r="H619" s="25" t="s">
-        <v>1271</v>
+        <v>1272</v>
       </c>
       <c r="I619" s="25" t="s">
-        <v>1271</v>
+        <v>1272</v>
       </c>
       <c r="J619" s="24"/>
       <c r="K619" s="24"/>
@@ -26306,7 +26312,7 @@
     </row>
     <row r="620" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A620" s="18" t="s">
-        <v>1272</v>
+        <v>1273</v>
       </c>
       <c r="B620" s="19">
         <v>1.04</v>
@@ -26322,13 +26328,13 @@
       </c>
       <c r="F620" s="23"/>
       <c r="G620" s="25" t="s">
-        <v>1273</v>
+        <v>1274</v>
       </c>
       <c r="H620" s="25" t="s">
-        <v>1273</v>
+        <v>1274</v>
       </c>
       <c r="I620" s="25" t="s">
-        <v>1273</v>
+        <v>1274</v>
       </c>
       <c r="J620" s="24"/>
       <c r="K620" s="25"/>
@@ -26339,7 +26345,7 @@
     </row>
     <row r="621" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A621" s="18" t="s">
-        <v>1274</v>
+        <v>1275</v>
       </c>
       <c r="B621" s="19">
         <v>2.1</v>
@@ -26354,13 +26360,13 @@
       <c r="F621" s="23"/>
       <c r="G621" s="24"/>
       <c r="H621" s="25" t="s">
-        <v>1275</v>
+        <v>1276</v>
       </c>
       <c r="I621" s="25" t="s">
-        <v>1275</v>
+        <v>1276</v>
       </c>
       <c r="J621" s="25" t="s">
-        <v>1275</v>
+        <v>1276</v>
       </c>
       <c r="K621" s="24"/>
       <c r="L621" s="24"/>
@@ -26370,7 +26376,7 @@
     </row>
     <row r="622" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A622" s="18" t="s">
-        <v>1276</v>
+        <v>1277</v>
       </c>
       <c r="B622" s="19">
         <v>2</v>
@@ -26385,7 +26391,7 @@
         <v>7.8</v>
       </c>
       <c r="F622" s="64" t="s">
-        <v>1277</v>
+        <v>1278</v>
       </c>
       <c r="G622" s="24"/>
       <c r="H622" s="24"/>
@@ -26399,7 +26405,7 @@
     </row>
     <row r="623" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A623" s="18" t="s">
-        <v>1278</v>
+        <v>1279</v>
       </c>
       <c r="B623" s="19">
         <v>2.11</v>
@@ -26415,10 +26421,10 @@
       </c>
       <c r="F623" s="23"/>
       <c r="G623" s="25" t="s">
-        <v>1278</v>
+        <v>1279</v>
       </c>
       <c r="H623" s="25" t="s">
-        <v>1278</v>
+        <v>1279</v>
       </c>
       <c r="I623" s="24"/>
       <c r="J623" s="24"/>
@@ -26430,7 +26436,7 @@
     </row>
     <row r="624" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A624" s="18" t="s">
-        <v>1279</v>
+        <v>1280</v>
       </c>
       <c r="B624" s="19">
         <v>2.7</v>
@@ -26443,16 +26449,16 @@
         <v>7.5</v>
       </c>
       <c r="F624" s="64" t="s">
-        <v>1280</v>
+        <v>1281</v>
       </c>
       <c r="G624" s="25" t="s">
-        <v>1280</v>
+        <v>1281</v>
       </c>
       <c r="H624" s="25" t="s">
-        <v>1280</v>
+        <v>1281</v>
       </c>
       <c r="I624" s="25" t="s">
-        <v>1280</v>
+        <v>1281</v>
       </c>
       <c r="J624" s="24"/>
       <c r="K624" s="24"/>
@@ -26463,7 +26469,7 @@
     </row>
     <row r="625" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A625" s="18" t="s">
-        <v>1281</v>
+        <v>1282</v>
       </c>
       <c r="B625" s="19" t="s">
         <v>29</v>
@@ -26477,7 +26483,7 @@
       <c r="E625" s="22"/>
       <c r="F625" s="27"/>
       <c r="G625" s="30" t="s">
-        <v>1282</v>
+        <v>1283</v>
       </c>
       <c r="H625" s="24"/>
       <c r="I625" s="24"/>
@@ -26490,7 +26496,7 @@
     </row>
     <row r="626" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A626" s="18" t="s">
-        <v>1283</v>
+        <v>1284</v>
       </c>
       <c r="B626" s="32">
         <v>2.56</v>
@@ -26499,22 +26505,22 @@
         <v>185</v>
       </c>
       <c r="D626" s="21" t="s">
-        <v>1284</v>
+        <v>1285</v>
       </c>
       <c r="E626" s="22">
         <v>7.2</v>
       </c>
       <c r="F626" s="27" t="s">
-        <v>1285</v>
+        <v>1286</v>
       </c>
       <c r="G626" s="25" t="s">
-        <v>1285</v>
+        <v>1286</v>
       </c>
       <c r="H626" s="25" t="s">
-        <v>1285</v>
+        <v>1286</v>
       </c>
       <c r="I626" s="25" t="s">
-        <v>1285</v>
+        <v>1286</v>
       </c>
       <c r="J626" s="24"/>
       <c r="K626" s="24"/>
@@ -26525,7 +26531,7 @@
     </row>
     <row r="627" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A627" s="18" t="s">
-        <v>1286</v>
+        <v>1287</v>
       </c>
       <c r="B627" s="19">
         <v>2.42</v>
@@ -26540,16 +26546,16 @@
         <v>7.9</v>
       </c>
       <c r="F627" s="27" t="s">
-        <v>1287</v>
+        <v>1288</v>
       </c>
       <c r="G627" s="25" t="s">
-        <v>1287</v>
+        <v>1288</v>
       </c>
       <c r="H627" s="25" t="s">
-        <v>1287</v>
+        <v>1288</v>
       </c>
       <c r="I627" s="25" t="s">
-        <v>1287</v>
+        <v>1288</v>
       </c>
       <c r="J627" s="24"/>
       <c r="K627" s="24"/>
@@ -26560,7 +26566,7 @@
     </row>
     <row r="628" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A628" s="18" t="s">
-        <v>1288</v>
+        <v>1289</v>
       </c>
       <c r="B628" s="19" t="s">
         <v>29</v>
@@ -26585,7 +26591,7 @@
     </row>
     <row r="629" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A629" s="18" t="s">
-        <v>1289</v>
+        <v>1290</v>
       </c>
       <c r="B629" s="19">
         <v>4.2</v>
@@ -26599,13 +26605,13 @@
       </c>
       <c r="F629" s="23"/>
       <c r="G629" s="25" t="s">
-        <v>1290</v>
+        <v>1291</v>
       </c>
       <c r="H629" s="25" t="s">
-        <v>1290</v>
+        <v>1291</v>
       </c>
       <c r="I629" s="25" t="s">
-        <v>1290</v>
+        <v>1291</v>
       </c>
       <c r="J629" s="24"/>
       <c r="K629" s="24"/>
@@ -26618,7 +26624,7 @@
     </row>
     <row r="630" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A630" s="18" t="s">
-        <v>1291</v>
+        <v>1292</v>
       </c>
       <c r="B630" s="19">
         <v>4.26</v>
@@ -26633,19 +26639,19 @@
         <v>8.5</v>
       </c>
       <c r="F630" s="27" t="s">
-        <v>1292</v>
+        <v>1293</v>
       </c>
       <c r="G630" s="57" t="s">
-        <v>1292</v>
+        <v>1293</v>
       </c>
       <c r="H630" s="57" t="s">
-        <v>1292</v>
+        <v>1293</v>
       </c>
       <c r="I630" s="59" t="s">
-        <v>1292</v>
+        <v>1293</v>
       </c>
       <c r="J630" s="57" t="s">
-        <v>1292</v>
+        <v>1293</v>
       </c>
       <c r="K630" s="24"/>
       <c r="L630" s="24"/>
@@ -26655,7 +26661,7 @@
     </row>
     <row r="631" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A631" s="18" t="s">
-        <v>1293</v>
+        <v>1294</v>
       </c>
       <c r="B631" s="19">
         <v>2.49</v>
@@ -26669,13 +26675,13 @@
       </c>
       <c r="F631" s="23"/>
       <c r="G631" s="25" t="s">
-        <v>1294</v>
+        <v>1295</v>
       </c>
       <c r="H631" s="25" t="s">
-        <v>1294</v>
+        <v>1295</v>
       </c>
       <c r="I631" s="25" t="s">
-        <v>1294</v>
+        <v>1295</v>
       </c>
       <c r="J631" s="24"/>
       <c r="K631" s="24"/>
@@ -26688,7 +26694,7 @@
     </row>
     <row r="632" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A632" s="18" t="s">
-        <v>1295</v>
+        <v>1296</v>
       </c>
       <c r="B632" s="19">
         <v>1.94</v>
@@ -26697,20 +26703,20 @@
         <v>18</v>
       </c>
       <c r="D632" s="21" t="s">
-        <v>1296</v>
+        <v>1297</v>
       </c>
       <c r="E632" s="22">
         <v>7.7</v>
       </c>
       <c r="F632" s="27"/>
       <c r="G632" s="25" t="s">
-        <v>1297</v>
+        <v>1298</v>
       </c>
       <c r="H632" s="25" t="s">
-        <v>1297</v>
+        <v>1298</v>
       </c>
       <c r="I632" s="25" t="s">
-        <v>1297</v>
+        <v>1298</v>
       </c>
       <c r="J632" s="24"/>
       <c r="K632" s="24"/>
@@ -26721,7 +26727,7 @@
     </row>
     <row r="633" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A633" s="18" t="s">
-        <v>1298</v>
+        <v>1299</v>
       </c>
       <c r="B633" s="19">
         <v>3.07</v>
@@ -26730,20 +26736,20 @@
         <v>185</v>
       </c>
       <c r="D633" s="21" t="s">
-        <v>1299</v>
+        <v>1300</v>
       </c>
       <c r="E633" s="22">
         <v>7.8</v>
       </c>
       <c r="F633" s="23"/>
       <c r="G633" s="25" t="s">
-        <v>1300</v>
+        <v>1301</v>
       </c>
       <c r="H633" s="25" t="s">
-        <v>1300</v>
+        <v>1301</v>
       </c>
       <c r="I633" s="25" t="s">
-        <v>1300</v>
+        <v>1301</v>
       </c>
       <c r="J633" s="24"/>
       <c r="K633" s="24"/>
@@ -26754,7 +26760,7 @@
     </row>
     <row r="634" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A634" s="18" t="s">
-        <v>1301</v>
+        <v>1302</v>
       </c>
       <c r="B634" s="19">
         <v>3.61</v>
@@ -26770,7 +26776,7 @@
       </c>
       <c r="F634" s="23"/>
       <c r="G634" s="25" t="s">
-        <v>1302</v>
+        <v>1303</v>
       </c>
       <c r="H634" s="24"/>
       <c r="I634" s="24"/>
@@ -26783,7 +26789,7 @@
     </row>
     <row r="635" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A635" s="18" t="s">
-        <v>1303</v>
+        <v>1304</v>
       </c>
       <c r="B635" s="19">
         <v>2.17</v>
@@ -26792,20 +26798,20 @@
         <v>172</v>
       </c>
       <c r="D635" s="21" t="s">
-        <v>1304</v>
+        <v>1305</v>
       </c>
       <c r="E635" s="22">
         <v>6.6</v>
       </c>
       <c r="F635" s="23"/>
       <c r="G635" s="57" t="s">
-        <v>1303</v>
+        <v>1304</v>
       </c>
       <c r="H635" s="25" t="s">
-        <v>1303</v>
+        <v>1304</v>
       </c>
       <c r="I635" s="25" t="s">
-        <v>1303</v>
+        <v>1304</v>
       </c>
       <c r="J635" s="24"/>
       <c r="K635" s="24"/>
@@ -26816,7 +26822,7 @@
     </row>
     <row r="636" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A636" s="18" t="s">
-        <v>1305</v>
+        <v>1306</v>
       </c>
       <c r="B636" s="19">
         <v>3.04</v>
@@ -26830,13 +26836,13 @@
       </c>
       <c r="F636" s="23"/>
       <c r="G636" s="25" t="s">
-        <v>1306</v>
+        <v>1307</v>
       </c>
       <c r="H636" s="25" t="s">
-        <v>1306</v>
+        <v>1307</v>
       </c>
       <c r="I636" s="25" t="s">
-        <v>1306</v>
+        <v>1307</v>
       </c>
       <c r="J636" s="24"/>
       <c r="K636" s="24"/>
@@ -27002,11 +27008,11 @@
     </row>
     <row r="646" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A646" s="18" t="s">
-        <v>1307</v>
+        <v>1308</v>
       </c>
       <c r="B646" s="19"/>
       <c r="C646" s="21" t="s">
-        <v>1308</v>
+        <v>1309</v>
       </c>
       <c r="D646" s="21"/>
       <c r="E646" s="22"/>
@@ -27023,7 +27029,7 @@
     </row>
     <row r="647" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A647" s="18" t="s">
-        <v>1309</v>
+        <v>1310</v>
       </c>
       <c r="B647" s="19">
         <v>2.16</v>
@@ -27035,13 +27041,13 @@
       <c r="E647" s="22"/>
       <c r="F647" s="23"/>
       <c r="G647" s="25" t="s">
-        <v>1309</v>
+        <v>1310</v>
       </c>
       <c r="H647" s="25" t="s">
-        <v>1309</v>
+        <v>1310</v>
       </c>
       <c r="I647" s="25" t="s">
-        <v>1309</v>
+        <v>1310</v>
       </c>
       <c r="J647" s="24"/>
       <c r="K647" s="24"/>
@@ -33818,16 +33824,16 @@
     </row>
     <row r="1046" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1046" t="s">
-        <v>1310</v>
+        <v>1311</v>
       </c>
       <c r="B1046" t="s">
         <v>29</v>
       </c>
       <c r="C1046" t="s">
-        <v>1311</v>
+        <v>1312</v>
       </c>
       <c r="D1046" t="s">
-        <v>1311</v>
+        <v>1312</v>
       </c>
       <c r="E1046">
         <v>0</v>
@@ -33835,16 +33841,16 @@
     </row>
     <row r="1047" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1047" t="s">
-        <v>1312</v>
+        <v>1313</v>
       </c>
       <c r="B1047" t="s">
         <v>29</v>
       </c>
       <c r="C1047" t="s">
-        <v>1311</v>
+        <v>1312</v>
       </c>
       <c r="D1047" t="s">
-        <v>1311</v>
+        <v>1312</v>
       </c>
       <c r="E1047">
         <v>0</v>
@@ -33852,16 +33858,16 @@
     </row>
     <row r="1048" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1048" t="s">
-        <v>1313</v>
+        <v>1314</v>
       </c>
       <c r="B1048" t="s">
         <v>29</v>
       </c>
       <c r="C1048" t="s">
-        <v>1311</v>
+        <v>1312</v>
       </c>
       <c r="D1048" t="s">
-        <v>1311</v>
+        <v>1312</v>
       </c>
       <c r="E1048">
         <v>0</v>
@@ -33869,7 +33875,7 @@
     </row>
     <row r="1049" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1049" t="s">
-        <v>1314</v>
+        <v>1315</v>
       </c>
       <c r="B1049" t="s">
         <v>29</v>
@@ -33878,7 +33884,7 @@
         <v>421</v>
       </c>
       <c r="D1049" t="s">
-        <v>1311</v>
+        <v>1312</v>
       </c>
       <c r="E1049">
         <v>0</v>
@@ -33886,7 +33892,7 @@
     </row>
     <row r="1050" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1050" t="s">
-        <v>1315</v>
+        <v>1316</v>
       </c>
       <c r="C1050" t="s">
         <v>421</v>
@@ -33894,26 +33900,34 @@
     </row>
     <row r="1051" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1051" t="s">
-        <v>1316</v>
+        <v>1317</v>
       </c>
       <c r="C1051" t="s">
-        <v>1317</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="1052" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1052" t="s">
+        <v>1319</v>
+      </c>
+      <c r="C1052" t="s">
         <v>1318</v>
-      </c>
-      <c r="C1052" t="s">
-        <v>1317</v>
       </c>
     </row>
     <row r="1053" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1053" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
       <c r="C1053" t="s">
         <v>185</v>
+      </c>
+    </row>
+    <row r="1054" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1054" t="s">
+        <v>1321</v>
+      </c>
+      <c r="C1054" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -34088,7 +34102,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="92" t="s">
-        <v>1320</v>
+        <v>1322</v>
       </c>
       <c r="B1" s="46"/>
     </row>
@@ -34098,10 +34112,10 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="46" t="s">
-        <v>1321</v>
+        <v>1323</v>
       </c>
       <c r="B3" s="46" t="s">
-        <v>1322</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -34118,10 +34132,10 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="46" t="s">
-        <v>1323</v>
+        <v>1325</v>
       </c>
       <c r="B6" s="46" t="s">
-        <v>1324</v>
+        <v>1326</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -34132,18 +34146,18 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="46" t="s">
-        <v>1325</v>
+        <v>1327</v>
       </c>
       <c r="B8" s="46" t="s">
-        <v>1326</v>
+        <v>1328</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="46" t="s">
-        <v>1327</v>
+        <v>1329</v>
       </c>
       <c r="B9" s="46" t="s">
-        <v>1328</v>
+        <v>1330</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -34160,10 +34174,10 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="46" t="s">
-        <v>1329</v>
+        <v>1331</v>
       </c>
       <c r="B12" s="46" t="s">
-        <v>1330</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -34180,10 +34194,10 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="46" t="s">
-        <v>1331</v>
+        <v>1333</v>
       </c>
       <c r="B15" s="46" t="s">
-        <v>1332</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -34243,7 +34257,7 @@
     </row>
     <row r="27" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B27" s="46" t="s">
-        <v>1333</v>
+        <v>1335</v>
       </c>
     </row>
   </sheetData>
@@ -34260,7 +34274,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="92" t="s">
-        <v>1320</v>
+        <v>1322</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -34268,126 +34282,126 @@
     </row>
     <row r="3" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B3" s="46" t="s">
-        <v>1334</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="46" t="s">
-        <v>1335</v>
+        <v>1337</v>
       </c>
       <c r="B4" s="46"/>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="46" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="46" t="s">
-        <v>1337</v>
+        <v>1339</v>
       </c>
       <c r="B6" s="46"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="46" t="s">
-        <v>1338</v>
+        <v>1340</v>
       </c>
       <c r="B7" s="46"/>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="46" t="s">
-        <v>1339</v>
+        <v>1341</v>
       </c>
       <c r="B8" s="46"/>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="46" t="s">
-        <v>1340</v>
+        <v>1342</v>
       </c>
       <c r="B9" s="46"/>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="46" t="s">
-        <v>1341</v>
+        <v>1343</v>
       </c>
       <c r="B10" s="46" t="s">
-        <v>1342</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="46" t="s">
-        <v>1343</v>
+        <v>1345</v>
       </c>
       <c r="B11" s="46"/>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="46" t="s">
-        <v>1344</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="46" t="s">
-        <v>1345</v>
+        <v>1347</v>
       </c>
       <c r="B13" s="46"/>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="46" t="s">
-        <v>1346</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="46" t="s">
-        <v>1347</v>
+        <v>1349</v>
       </c>
       <c r="B15" s="46"/>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="46" t="s">
-        <v>1348</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="46" t="s">
-        <v>1349</v>
+        <v>1351</v>
       </c>
       <c r="B17" s="46"/>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="46" t="s">
-        <v>1350</v>
+        <v>1352</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="46" t="s">
-        <v>1351</v>
+        <v>1353</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="46" t="s">
-        <v>1352</v>
+        <v>1354</v>
       </c>
       <c r="B20" s="46"/>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="46" t="s">
-        <v>1353</v>
+        <v>1355</v>
       </c>
       <c r="B21" s="46"/>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="46" t="s">
-        <v>1354</v>
+        <v>1356</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="46" t="s">
-        <v>1355</v>
+        <v>1357</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="46" t="s">
-        <v>1356</v>
+        <v>1358</v>
       </c>
     </row>
   </sheetData>

</xml_diff>